<commit_message>
Resolve merge conflict and update README and requirements
</commit_message>
<xml_diff>
--- a/data/raw/forms/Filled Abstract Forms.xlsx
+++ b/data/raw/forms/Filled Abstract Forms.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ksarawgi\OneDrive - IMC Construction, Inc\Owner Contracts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incyte-my.sharepoint.com/personal/c250479_incyte_com/Documents/Documents/Projects/IMC-Contract-Intelligence-Assistant/data/raw/forms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6C3F98A-C4E2-4A8A-9D3E-B4C2590CF707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{B6C3F98A-C4E2-4A8A-9D3E-B4C2590CF707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E416F4A0-722C-466A-97B3-2C2FF99B818E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="21825" yWindow="5475" windowWidth="32400" windowHeight="16860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Form1" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <definedName name="_56F9DC9755BA473782653E2940F9SourceDocId">"{bba344bd-0d21-46cb-9be1-bf9c2d276fef}"</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2928" uniqueCount="1316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2953" uniqueCount="1340">
   <si>
     <t>ID</t>
   </si>
@@ -5408,7 +5409,79 @@
     <t>{bba344bd-0d21-46cb-9be1-bf9c2d276fef}</t>
   </si>
   <si>
-    <t>UID</t>
+    <t>Contract__1.pdf</t>
+  </si>
+  <si>
+    <t>Contract file names</t>
+  </si>
+  <si>
+    <t>Contract__2.pdf</t>
+  </si>
+  <si>
+    <t>Contract__3.pdf</t>
+  </si>
+  <si>
+    <t>Contract__4.pdf</t>
+  </si>
+  <si>
+    <t>Contract__5.pdf</t>
+  </si>
+  <si>
+    <t>Contract__6.pdf</t>
+  </si>
+  <si>
+    <t>Contract__7.pdf</t>
+  </si>
+  <si>
+    <t>Contract__8.pdf</t>
+  </si>
+  <si>
+    <t>Contract__17.pdf</t>
+  </si>
+  <si>
+    <t>Contract__18.pdf</t>
+  </si>
+  <si>
+    <t>Contract__9.pdf</t>
+  </si>
+  <si>
+    <t>Contract__10.pdf</t>
+  </si>
+  <si>
+    <t>Contract__11.pdf</t>
+  </si>
+  <si>
+    <t>Contract__19.pdf</t>
+  </si>
+  <si>
+    <t>Contract__20.pdf</t>
+  </si>
+  <si>
+    <t>Contract__21.pdf</t>
+  </si>
+  <si>
+    <t>Contract__12.pdf</t>
+  </si>
+  <si>
+    <t>Contract__22.pdf</t>
+  </si>
+  <si>
+    <t>Contract__13.pdf</t>
+  </si>
+  <si>
+    <t>Contract__14.pdf</t>
+  </si>
+  <si>
+    <t>Contract__23.pdf</t>
+  </si>
+  <si>
+    <t>Contract__24.pdf</t>
+  </si>
+  <si>
+    <t>Contract__16.pdf</t>
+  </si>
+  <si>
+    <t>Contract__25.pdf</t>
   </si>
 </sst>
 </file>
@@ -5856,828 +5929,140 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="B1:DU28" totalsRowShown="0">
   <autoFilter ref="B1:DU28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="124">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="123">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="id"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="What is the Execution Date of the Contract Agreement?" dataDxfId="122">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r7d90da3b6d0d4d5ab58194bafa660753"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="What is the AIA Form of Contract Agreement?" dataDxfId="121">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r333878a557e64604a2416d5356acb191"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="What is the Contract Type for this Project? (Custom Text Answer)" dataDxfId="120">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r20892b4c7cd44a4ab993418747b11a00"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Are there Consequential Damages on the Project?" dataDxfId="119">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r31f357e6c7814e978a1190d0dea30125"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="What are the are the Consequential Damages Terms &amp; Conditions?" dataDxfId="118">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r13b23d7a98b24697833e7b4706ee64df"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Is there a mutual waiver of Consequential Damages in the Contract?" dataDxfId="117">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r0dd5ea5075534da8adc5163fc641e754"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Are there Liquidated Damages on the Project?" dataDxfId="116">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="ra0b8f43bd5a0458397bca3de86c47df1"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="What are the are the Liquidated Damages Terms &amp; Conditions?" dataDxfId="115">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rcb39888485954b849ec25be717540429"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="123"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="What is the Execution Date of the Contract Agreement?" dataDxfId="122"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="What is the AIA Form of Contract Agreement?" dataDxfId="121"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="What is the Contract Type for this Project? (Custom Text Answer)" dataDxfId="120"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Are there Consequential Damages on the Project?" dataDxfId="119"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="What are the are the Consequential Damages Terms &amp; Conditions?" dataDxfId="118"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Is there a mutual waiver of Consequential Damages in the Contract?" dataDxfId="117"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Are there Liquidated Damages on the Project?" dataDxfId="116"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="What are the are the Liquidated Damages Terms &amp; Conditions?" dataDxfId="115"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="What is the Article # for Consequential &amp; Liquidated Damages?" dataDxfId="114"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="What is the CCIP Rate % for this Project?" dataDxfId="113">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r75c08cbdffb9486eba28ecf67b79f977"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Is IMC or the Owner carrying the Builder's Risk Policy for this project?" dataDxfId="112">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rf250282fa9f047f292532a1f38dd6422"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="What is the Builders Risk %?" dataDxfId="111">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r68c6e076211347e6b7373b3eabe809fa"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="What is the Builders Risk Deductible? ($)" dataDxfId="110">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r50d5dcc2b0b8467cbfa057ae78eb727b"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="What is the Builders Risk Waiver of Subrogation Appendix / Exhibit (Letter or Number) if the Owner Carries the Policy" dataDxfId="109">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r64b0f1d30e4043d1b039a10f86a00c06"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Is Professional Liability Insurance Required for this project?" dataDxfId="108">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rb29a12d680724ea7a57805d41ba7a872"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Is Railroad Insurance Required for this project?" dataDxfId="107">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rfbb7e9f167b94f2092dc0076844d8ba5"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Is Pollution Liability Insurance Required for this project?" dataDxfId="106">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r98a6045c74294501a236c2d58930a2d1"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Is a Payment &amp; Performance Bond Required for this project?" dataDxfId="105">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r5a009cdb311b4b30bc983bcd6a2c5063"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="What is the CCIP Rate % for this Project?" dataDxfId="113"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Is IMC or the Owner carrying the Builder's Risk Policy for this project?" dataDxfId="112"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="What is the Builders Risk %?" dataDxfId="111"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="What is the Builders Risk Deductible? ($)" dataDxfId="110"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="What is the Builders Risk Waiver of Subrogation Appendix / Exhibit (Letter or Number) if the Owner Carries the Policy" dataDxfId="109"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Is Professional Liability Insurance Required for this project?" dataDxfId="108"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Is Railroad Insurance Required for this project?" dataDxfId="107"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Is Pollution Liability Insurance Required for this project?" dataDxfId="106"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Is a Payment &amp; Performance Bond Required for this project?" dataDxfId="105"/>
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="What is the Payment &amp; Performance Bond Article #?" dataDxfId="104"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="What are the Payment &amp; Performance Bond Article Terms &amp; Conditions?" dataDxfId="103">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r3aefc1d090a74439b684bb4b245b2177"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="What are the Payment &amp; Performance Bond Article Terms &amp; Conditions?" dataDxfId="103"/>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="What is the Contract Documents Definition &amp; Incorporation Article #?" dataDxfId="102"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="What are the Contract Documents Definition &amp; Incorporation Definitions, Terms, &amp; Conditions?" dataDxfId="101">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r3e1f9ae94afa448a9418b710cb752f34"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="What are the Contract Documents Definition &amp; Incorporation Definitions, Terms, &amp; Conditions?" dataDxfId="101"/>
     <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="What is the IMC Design Document Review obligations Article #?" dataDxfId="100"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="What are the Terms &amp; Conditions / IMC's obligations for Design Document Review?" dataDxfId="99">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r8f48763501c141cabcba9ccb9f7387b8"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="What are the Terms &amp; Conditions / IMC's obligations for Design Document Review?" dataDxfId="99"/>
     <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="What is the Submittal Alternates, Substitutions, &amp; Contract Document Deviations Article #?" dataDxfId="98"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="What are the Submittal Alternates, Substitutions, &amp; Contract Document Deviations Terms &amp; Conditions?" dataDxfId="97">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r511f20b7ad754365b8911145766f7d2c"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Do we have a Precon Agreement?" dataDxfId="96">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r99a0cc669ecc4fdfba741c1754b46757"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Is Precon Reimbursable beyond the Agreement?" dataDxfId="95">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r91aa4272d0e8428ab83090d2151968e1"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="What are the Submittal Alternates, Substitutions, &amp; Contract Document Deviations Terms &amp; Conditions?" dataDxfId="97"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Do we have a Precon Agreement?" dataDxfId="96"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Is Precon Reimbursable beyond the Agreement?" dataDxfId="95"/>
     <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="What is the Precon Reimbursable Contract Article #?" dataDxfId="94"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="What are the Precon Reimbursable Terms &amp; Conditions?" dataDxfId="93">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r421f93c42ecd4034968430d5904a832d"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="What are the Precon Reimbursable Terms &amp; Conditions?" dataDxfId="93"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="What is the Subcontractor Bid Requirements Article #?" dataDxfId="92"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Are the Subcontractor Bids / Bid Tabs Required to be Provided to Owner?" dataDxfId="91">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="re5de246da8c448649597351cc4ac3e63"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="What is the Subcontractor Required Number of Bids per package?" dataDxfId="90">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rddb08ff6ba1a4f22801cbd84cd68b9ff"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Are the Subcontractor Bids / Bid Tabs Required to be Provided to Owner?" dataDxfId="91"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="What is the Subcontractor Required Number of Bids per package?" dataDxfId="90"/>
     <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="What are the Subcontractor Bids / Bid Tabs Provided to Owner Terms &amp; Conditions?" dataDxfId="89"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="Does a Subcontractor Award have to be Approved by Owner?" dataDxfId="88">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r88d51b5c8aad479d846e9270635a68dd"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="Can Owner Mandate Specific Subcontractors be used?" dataDxfId="87">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r71eec1ad3095454489076c8df8dd6f2d"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="Is IMC Entitled a PCCO for Owner Selected / Mandated Subcontractors?" dataDxfId="86">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="re8020cd41e464042bec4618f513425f6"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="Does a Subcontractor Award have to be Approved by Owner?" dataDxfId="88"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="Can Owner Mandate Specific Subcontractors be used?" dataDxfId="87"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="Is IMC Entitled a PCCO for Owner Selected / Mandated Subcontractors?" dataDxfId="86"/>
     <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="What is the GMP Shared Savings Article #?" dataDxfId="85"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="What are the GMP Shared Savings Terms &amp; Conditions?" dataDxfId="84">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r2c27a4dfe6254b67a6a612103e619369"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="What are the GMP Shared Savings Terms &amp; Conditions?" dataDxfId="84"/>
     <tableColumn id="48" xr3:uid="{00000000-0010-0000-0000-000030000000}" name="What is the GMP Buyout Savings Article #?" dataDxfId="83"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="Do GMP Buyout Savings need to be Reported to Owner?" dataDxfId="82">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="ref2cc6ee8621439892c97520c392e379"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0000-000032000000}" name="Must the GMP Buyout Savings be Shown on Monthly Schedule of Values?" dataDxfId="81">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r04c110c6f3904c37894eec3af1b6f577"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0000-000033000000}" name="What are the GMP Buyout Savings Definition &amp; Terms &amp; Conditions?" dataDxfId="80">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r0e8520abe8c34ec0b67941171a4f7ad3"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0000-000034000000}" name="Must Use of Buyout Savings for Trade Costs be Approved by Owner?" dataDxfId="79">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r219eb35008dd426db1f843a8ca13cd40"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0000-000035000000}" name="What is the General Conditions Rate Sheet Appendix / Exhibit (A,B,C,D, Etc.)?" dataDxfId="78">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r1e4222322f8a4b3290b5994aa0c4d432"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0000-000036000000}" name="What is the General Conditions Rate Sheet Year?" dataDxfId="77">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r3f1689564d114dc1a62c0287b4a19e3f"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0000-000031000000}" name="Do GMP Buyout Savings need to be Reported to Owner?" dataDxfId="82"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0000-000032000000}" name="Must the GMP Buyout Savings be Shown on Monthly Schedule of Values?" dataDxfId="81"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0000-000033000000}" name="What are the GMP Buyout Savings Definition &amp; Terms &amp; Conditions?" dataDxfId="80"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0000-000034000000}" name="Must Use of Buyout Savings for Trade Costs be Approved by Owner?" dataDxfId="79"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0000-000035000000}" name="What is the General Conditions Rate Sheet Appendix / Exhibit (A,B,C,D, Etc.)?" dataDxfId="78"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0000-000036000000}" name="What is the General Conditions Rate Sheet Year?" dataDxfId="77"/>
     <tableColumn id="55" xr3:uid="{00000000-0010-0000-0000-000037000000}" name="What is the Cost of the Work Article #?" dataDxfId="76"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0000-000038000000}" name="What is the definition for the Cost of the Work?" dataDxfId="75">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="red658e215a034f4a9b4e4d0669b99d64"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0000-000038000000}" name="What is the definition for the Cost of the Work?" dataDxfId="75"/>
     <tableColumn id="57" xr3:uid="{00000000-0010-0000-0000-000039000000}" name="What is the Contingency Usage Article #?" dataDxfId="74"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0000-00003A000000}" name="What are the Contingency Usage Terms and Conditions?" dataDxfId="73">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="re35f6e8c39504df5a53ab299d2c75388"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0000-00003B000000}" name="What are the Contingency Usage Owner Notification Requirements?" dataDxfId="72">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rc8125195f5784cd0bcbe5834f31ba726"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0000-00003C000000}" name="What is the General Conditions Type?" dataDxfId="71">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r603600d87fc5401c8e50b4b82ee0e1b4"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0000-00003D000000}" name="What are the General Conditions Billing Backup Requirements?" dataDxfId="70">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r234a80e39db04a179f4e69d1f7f8305a"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0000-00003E000000}" name="Are there General Conditions / Requirements Owner Audit Provisions?" dataDxfId="69">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r1aef87de3aaa46b292efd902412fb1db"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0000-00003F000000}" name="What is the definition of General Conditions for this project? (01 v 50 Code Split)" dataDxfId="68">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r6b642609bbd2483496535f5ea4426402"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0000-000040000000}" name="What is the Change Markup - Subcontractor %?" dataDxfId="67">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r53ef0168697245aea3523acf623b5b6e"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0000-000041000000}" name="What is the Change Markup - Tiered Subcontractor %?" dataDxfId="66">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r16fbd2d0ede144398dc1d38017db246f"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0000-000042000000}" name="What is the Change Markup - IMC Fee %?" dataDxfId="65">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r94b71574e77144a9944acab61e704546"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0000-000043000000}" name="What is the Change Markup - CCIP %?" dataDxfId="64">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r4ee458eeafc24c60981e7abfa3f60afc"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0000-000044000000}" name="What is the Change Markup - Warranty %?" dataDxfId="63">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rc8a478ec1f45406a9068cf17f0e292d9"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0000-000045000000}" name="What is the Change Markup - General Conditions %?" dataDxfId="62">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r36e4d147820949b0a778dc56a7b1b9d6"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0000-000046000000}" name="What is the Change Markup - CM Insurance %?" dataDxfId="61">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r765d687918fb4bd388cd9593d18256bf"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0000-000047000000}" name="What is the Change Markup - P &amp; P Bond %?" dataDxfId="60">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r79ec9c8349034fa19d9d4e7174300ef8"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0000-00003A000000}" name="What are the Contingency Usage Terms and Conditions?" dataDxfId="73"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0000-00003B000000}" name="What are the Contingency Usage Owner Notification Requirements?" dataDxfId="72"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0000-00003C000000}" name="What is the General Conditions Type?" dataDxfId="71"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0000-00003D000000}" name="What are the General Conditions Billing Backup Requirements?" dataDxfId="70"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0000-00003E000000}" name="Are there General Conditions / Requirements Owner Audit Provisions?" dataDxfId="69"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0000-00003F000000}" name="What is the definition of General Conditions for this project? (01 v 50 Code Split)" dataDxfId="68"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0000-000040000000}" name="What is the Change Markup - Subcontractor %?" dataDxfId="67"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0000-000041000000}" name="What is the Change Markup - Tiered Subcontractor %?" dataDxfId="66"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0000-000042000000}" name="What is the Change Markup - IMC Fee %?" dataDxfId="65"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0000-000043000000}" name="What is the Change Markup - CCIP %?" dataDxfId="64"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0000-000044000000}" name="What is the Change Markup - Warranty %?" dataDxfId="63"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0000-000045000000}" name="What is the Change Markup - General Conditions %?" dataDxfId="62"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0000-000046000000}" name="What is the Change Markup - CM Insurance %?" dataDxfId="61"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0000-000047000000}" name="What is the Change Markup - P &amp; P Bond %?" dataDxfId="60"/>
     <tableColumn id="72" xr3:uid="{00000000-0010-0000-0000-000048000000}" name="What is the Adverse Weather Days Article #?" dataDxfId="59"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0000-000049000000}" name="What are the Adverse Weather Days Terms &amp; Conditions?" dataDxfId="58">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r2762b1bd4a7e46ee8aea16ea651f08cb"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0000-00004A000000}" name="Within how many days must we notify the owner of adverse weather day impacts?" dataDxfId="57">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rb7970e13cb2c4da085a4bde4a67b4cf5"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0000-00004B000000}" name="How many Adverse Weather Days Included in Contract Agreement?" dataDxfId="56">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r8cd57f4b8b7c4f3e9383f6cc22643e5f"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0000-000049000000}" name="What are the Adverse Weather Days Terms &amp; Conditions?" dataDxfId="58"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0000-00004A000000}" name="Within how many days must we notify the owner of adverse weather day impacts?" dataDxfId="57"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0000-00004B000000}" name="How many Adverse Weather Days Included in Contract Agreement?" dataDxfId="56"/>
     <tableColumn id="76" xr3:uid="{00000000-0010-0000-0000-00004C000000}" name="What is the Schedule Requirements Article #?" dataDxfId="55"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0000-00004D000000}" name="What are the Schedule Requirements Terms &amp; Conditions?" dataDxfId="54">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r9222b568c0764e8b9f86561d7612dc80"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0000-00004D000000}" name="What are the Schedule Requirements Terms &amp; Conditions?" dataDxfId="54"/>
     <tableColumn id="78" xr3:uid="{00000000-0010-0000-0000-00004E000000}" name="What is the Daily Log &amp; Manpower Article #?" dataDxfId="53"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0000-00004F000000}" name="What are the Daily Log &amp; Manpower Terms and Conditions?" dataDxfId="52">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r91aacfed7c034922963019a3a708273e"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0000-00004F000000}" name="What are the Daily Log &amp; Manpower Terms and Conditions?" dataDxfId="52"/>
     <tableColumn id="80" xr3:uid="{00000000-0010-0000-0000-000050000000}" name="What is the Schedule Delay / Time Issues Article #?" dataDxfId="51"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0000-000051000000}" name="What are the Schedule Delay / Time Issues Terms &amp; Conditions?" dataDxfId="50">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r61e13bffea00487a89561a5286eddd70"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0000-000052000000}" name="How much Schedule Delay / Time Issues Notice to Owner Requirements (Within What # of Days)?" dataDxfId="49">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r1ba7d730cb1d45cfb45f41fdd8d3f726"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0000-000051000000}" name="What are the Schedule Delay / Time Issues Terms &amp; Conditions?" dataDxfId="50"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0000-000052000000}" name="How much Schedule Delay / Time Issues Notice to Owner Requirements (Within What # of Days)?" dataDxfId="49"/>
     <tableColumn id="83" xr3:uid="{00000000-0010-0000-0000-000053000000}" name="What is the Schedule Acceleration Directed by Owner Article #?" dataDxfId="48"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0000-000054000000}" name="What are the Schedule Acceleration Directed by Owner Terms &amp; Conditions?" dataDxfId="47">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rb9f3e9f03f824bac8b97ad79309b8b80"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0000-000055000000}" name="What are the Schedule Definitions of Days (Work / Calendar / Holidays / Etc.)?" dataDxfId="46">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rccc43ba04ce8481d82e5bbfa65d5efc8"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0000-000056000000}" name="What is the Substantial Completion Article #?" dataDxfId="45">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r71be6f0b174849f0b3c027cae6320fed"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0000-000057000000}" name="What are the Substantial Completion Terms &amp; Conditions?" dataDxfId="44">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r6a2252e44d17494baf7280077a8d7048"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="88" xr3:uid="{00000000-0010-0000-0000-000058000000}" name="What is the Final Completion Definition Article #?" dataDxfId="43">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="ra94986dd41e9411786bd6a9547d5dce9"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="89" xr3:uid="{00000000-0010-0000-0000-000059000000}" name="What is the Final Completion Definition?" dataDxfId="42">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r7506d7a2568f4cbc801da6dfd331073b"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="90" xr3:uid="{00000000-0010-0000-0000-00005A000000}" name="Are there Project Interim Milestones?" dataDxfId="41">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="raa0a22f6e8c843569c9f103702978d9c"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="91" xr3:uid="{00000000-0010-0000-0000-00005B000000}" name="Project Interim Milestones List" dataDxfId="40">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r651c21d8cd044857bc5d4c2e6f1f15f7"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="92" xr3:uid="{00000000-0010-0000-0000-00005C000000}" name="What is the Payment Terms (Progress &amp; Final) Article #?" dataDxfId="39">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r62018dadbca944eb8e13d572a5e25a92"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="93" xr3:uid="{00000000-0010-0000-0000-00005D000000}" name="What are the Payment Terms Retainage %?" dataDxfId="38">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r7c3dc7565df04de5a818045f10cebda4"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="94" xr3:uid="{00000000-0010-0000-0000-00005E000000}" name="What is the Payment Terms for Retainage Reduction Article #?" dataDxfId="37">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r86c1b7203b3443f3be9c09a62ec8a2dd"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="95" xr3:uid="{00000000-0010-0000-0000-00005F000000}" name="What are the Payment Terms &amp; Conditions for Retainage Reduction?" dataDxfId="36">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r61312d8a3bf241b595a8a7cea92d7d7c"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="96" xr3:uid="{00000000-0010-0000-0000-000060000000}" name="Are there Payment Terms for Retainage on General Conditions?" dataDxfId="35">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rbd05295cc26a4fdd89fed946070ef8fc"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="97" xr3:uid="{00000000-0010-0000-0000-000061000000}" name="Are there Payment Terms for Retainage on Fee?" dataDxfId="34">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r79d8d8378ee14f61a0aca947618aa45e"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0000-000054000000}" name="What are the Schedule Acceleration Directed by Owner Terms &amp; Conditions?" dataDxfId="47"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0000-000055000000}" name="What are the Schedule Definitions of Days (Work / Calendar / Holidays / Etc.)?" dataDxfId="46"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0000-000056000000}" name="What is the Substantial Completion Article #?" dataDxfId="45"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0000-000057000000}" name="What are the Substantial Completion Terms &amp; Conditions?" dataDxfId="44"/>
+    <tableColumn id="88" xr3:uid="{00000000-0010-0000-0000-000058000000}" name="What is the Final Completion Definition Article #?" dataDxfId="43"/>
+    <tableColumn id="89" xr3:uid="{00000000-0010-0000-0000-000059000000}" name="What is the Final Completion Definition?" dataDxfId="42"/>
+    <tableColumn id="90" xr3:uid="{00000000-0010-0000-0000-00005A000000}" name="Are there Project Interim Milestones?" dataDxfId="41"/>
+    <tableColumn id="91" xr3:uid="{00000000-0010-0000-0000-00005B000000}" name="Project Interim Milestones List" dataDxfId="40"/>
+    <tableColumn id="92" xr3:uid="{00000000-0010-0000-0000-00005C000000}" name="What is the Payment Terms (Progress &amp; Final) Article #?" dataDxfId="39"/>
+    <tableColumn id="93" xr3:uid="{00000000-0010-0000-0000-00005D000000}" name="What are the Payment Terms Retainage %?" dataDxfId="38"/>
+    <tableColumn id="94" xr3:uid="{00000000-0010-0000-0000-00005E000000}" name="What is the Payment Terms for Retainage Reduction Article #?" dataDxfId="37"/>
+    <tableColumn id="95" xr3:uid="{00000000-0010-0000-0000-00005F000000}" name="What are the Payment Terms &amp; Conditions for Retainage Reduction?" dataDxfId="36"/>
+    <tableColumn id="96" xr3:uid="{00000000-0010-0000-0000-000060000000}" name="Are there Payment Terms for Retainage on General Conditions?" dataDxfId="35"/>
+    <tableColumn id="97" xr3:uid="{00000000-0010-0000-0000-000061000000}" name="Are there Payment Terms for Retainage on Fee?" dataDxfId="34"/>
     <tableColumn id="98" xr3:uid="{00000000-0010-0000-0000-000062000000}" name="What is the Payment Terms for Offsite Stored Material Article #?" dataDxfId="33"/>
-    <tableColumn id="99" xr3:uid="{00000000-0010-0000-0000-000063000000}" name="What are the Terms and Conditions for Payment of Offsite Stored Material?" dataDxfId="32">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rcf60812b97f642489be7187347eecf59"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="100" xr3:uid="{00000000-0010-0000-0000-000064000000}" name="How many days within Approved Application for Owner Payment?" dataDxfId="31">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r69ddd5267a474d7fbf1ef4a31f0b343a"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="101" xr3:uid="{00000000-0010-0000-0000-000065000000}" name="What is the Article # for IMC's Stop Work Ability for late Owner payment?" dataDxfId="30">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r7befd93a2b044ddcb732af34021a7d68"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="102" xr3:uid="{00000000-0010-0000-0000-000066000000}" name="What are the Terms &amp; Conditions for IMC's Stop Work Ability for late Owner payment?" dataDxfId="29">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r1150fbd8e5ce40bd9ae6b4d3aca9c087"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="103" xr3:uid="{00000000-0010-0000-0000-000067000000}" name="What is the Dispute Resolution Article #?" dataDxfId="28">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r6096f99c96944892a8742a600d7a25c9"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="104" xr3:uid="{00000000-0010-0000-0000-000068000000}" name="What is the CM Suspension / Termination Article #?" dataDxfId="27">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rbc70f0e67c2546ce991f8ceda7d12e27"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="105" xr3:uid="{00000000-0010-0000-0000-000069000000}" name="How many days notice must the Owner give IMC for CM Termination for Convenience?" dataDxfId="26">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r2b239e19bc72478f9703cfb6ea697743"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="106" xr3:uid="{00000000-0010-0000-0000-00006A000000}" name="How many days notice must the Owner give IMC for CM Termination for Cause?" dataDxfId="25">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r55ecd76cb2f8456c86d9f98841c17b1f"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="99" xr3:uid="{00000000-0010-0000-0000-000063000000}" name="What are the Terms and Conditions for Payment of Offsite Stored Material?" dataDxfId="32"/>
+    <tableColumn id="100" xr3:uid="{00000000-0010-0000-0000-000064000000}" name="How many days within Approved Application for Owner Payment?" dataDxfId="31"/>
+    <tableColumn id="101" xr3:uid="{00000000-0010-0000-0000-000065000000}" name="What is the Article # for IMC's Stop Work Ability for late Owner payment?" dataDxfId="30"/>
+    <tableColumn id="102" xr3:uid="{00000000-0010-0000-0000-000066000000}" name="What are the Terms &amp; Conditions for IMC's Stop Work Ability for late Owner payment?" dataDxfId="29"/>
+    <tableColumn id="103" xr3:uid="{00000000-0010-0000-0000-000067000000}" name="What is the Dispute Resolution Article #?" dataDxfId="28"/>
+    <tableColumn id="104" xr3:uid="{00000000-0010-0000-0000-000068000000}" name="What is the CM Suspension / Termination Article #?" dataDxfId="27"/>
+    <tableColumn id="105" xr3:uid="{00000000-0010-0000-0000-000069000000}" name="How many days notice must the Owner give IMC for CM Termination for Convenience?" dataDxfId="26"/>
+    <tableColumn id="106" xr3:uid="{00000000-0010-0000-0000-00006A000000}" name="How many days notice must the Owner give IMC for CM Termination for Cause?" dataDxfId="25"/>
     <tableColumn id="107" xr3:uid="{00000000-0010-0000-0000-00006B000000}" name="What is the Direct Negotiation Duration (# of Days)?" dataDxfId="24"/>
     <tableColumn id="108" xr3:uid="{00000000-0010-0000-0000-00006C000000}" name="What is the Mediation Duration (# of Days)?" dataDxfId="23"/>
     <tableColumn id="109" xr3:uid="{00000000-0010-0000-0000-00006D000000}" name="What is the Mediator Selection Duration (# of Days)?" dataDxfId="22"/>
     <tableColumn id="110" xr3:uid="{00000000-0010-0000-0000-00006E000000}" name="How many days after Mediator Selection is the Mediation Session?" dataDxfId="21"/>
     <tableColumn id="111" xr3:uid="{00000000-0010-0000-0000-00006F000000}" name="What is the Warranty Terms &amp; Conditions Article #?" dataDxfId="20"/>
-    <tableColumn id="112" xr3:uid="{00000000-0010-0000-0000-000070000000}" name="What are the Warranty Terms &amp; Conditions?" dataDxfId="19">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r216255fe8cbc4d08ab0109f4de1d61b7"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="112" xr3:uid="{00000000-0010-0000-0000-000070000000}" name="What are the Warranty Terms &amp; Conditions?" dataDxfId="19"/>
     <tableColumn id="113" xr3:uid="{00000000-0010-0000-0000-000071000000}" name="What is the As-Built / Record Documents Requirements Article #?" dataDxfId="18"/>
-    <tableColumn id="114" xr3:uid="{00000000-0010-0000-0000-000072000000}" name="What are the As-Built / Record Documents Requirements?" dataDxfId="17">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r123dd14384f449e0ae91d811f71dad3e"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="115" xr3:uid="{00000000-0010-0000-0000-000073000000}" name="What is the Final Payment Article #?" dataDxfId="16">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r665a7ea397a34d568aac3d8e8420000f"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="116" xr3:uid="{00000000-0010-0000-0000-000074000000}" name="What are the Final Payment Terms &amp; Conditions?" dataDxfId="15">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r9649ee9242b2466f860eab1f1ab1ec69"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="114" xr3:uid="{00000000-0010-0000-0000-000072000000}" name="What are the As-Built / Record Documents Requirements?" dataDxfId="17"/>
+    <tableColumn id="115" xr3:uid="{00000000-0010-0000-0000-000073000000}" name="What is the Final Payment Article #?" dataDxfId="16"/>
+    <tableColumn id="116" xr3:uid="{00000000-0010-0000-0000-000074000000}" name="What are the Final Payment Terms &amp; Conditions?" dataDxfId="15"/>
     <tableColumn id="117" xr3:uid="{00000000-0010-0000-0000-000075000000}" name="What is the Concealed / Unknown / Hazardous Conditions Article #?" dataDxfId="14"/>
-    <tableColumn id="118" xr3:uid="{00000000-0010-0000-0000-000076000000}" name="What are the Concealed / Unknown / Hazardous Conditions Terms &amp; Conditions?" dataDxfId="13">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r4bbab4541b2847df9ac326d5844756d5"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="119" xr3:uid="{00000000-0010-0000-0000-000077000000}" name="How much Concealed / Unknown / Hazardous Conditions Notice to Owner Requirements (Within What # of Days)?" dataDxfId="12">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rf87b2a6e53a644849cfb2d142aa857d2"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="120" xr3:uid="{00000000-0010-0000-0000-000078000000}" name="List the Owner / Project Required Reports" dataDxfId="11">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rf51502d08e1f4893832e976c8314d940"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="121" xr3:uid="{00000000-0010-0000-0000-000079000000}" name="Is Owner Allowed to Occupy Building Prior to Substantial Completion Article?" dataDxfId="10">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r5d645ce804e343f289e48c56f820ade9"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="118" xr3:uid="{00000000-0010-0000-0000-000076000000}" name="What are the Concealed / Unknown / Hazardous Conditions Terms &amp; Conditions?" dataDxfId="13"/>
+    <tableColumn id="119" xr3:uid="{00000000-0010-0000-0000-000077000000}" name="How much Concealed / Unknown / Hazardous Conditions Notice to Owner Requirements (Within What # of Days)?" dataDxfId="12"/>
+    <tableColumn id="120" xr3:uid="{00000000-0010-0000-0000-000078000000}" name="List the Owner / Project Required Reports" dataDxfId="11"/>
+    <tableColumn id="121" xr3:uid="{00000000-0010-0000-0000-000079000000}" name="Is Owner Allowed to Occupy Building Prior to Substantial Completion Article?" dataDxfId="10"/>
     <tableColumn id="122" xr3:uid="{00000000-0010-0000-0000-00007A000000}" name="If the Owner is Allowed to Occupy Building Prior to Substantial Completion, what is the Article #?" dataDxfId="9"/>
-    <tableColumn id="123" xr3:uid="{00000000-0010-0000-0000-00007B000000}" name="Hazardous Materials - IMC is Only Responsible Content Created by Us or our Subcontractors" dataDxfId="8">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rc2901229e6604efb8202cde185cec144"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="124" xr3:uid="{00000000-0010-0000-0000-00007C000000}" name="Hazardous Materials - IMC is Entitled to Stop Work, and Recover Cost for Delay for_x000a_  Encountered Hazardous Material" dataDxfId="7">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rbbec339b56db4500836dd7699a6a717e"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="125" xr3:uid="{00000000-0010-0000-0000-00007D000000}" name="What is the Labor?" dataDxfId="6">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r88c463a257ca4ac591b3b83ba8b5e495"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="126" xr3:uid="{00000000-0010-0000-0000-00007E000000}" name="Is IMC Responsible to Recover Delay (Cost &amp; Schedule) for labor related work stoppage;_x000a_  strike etc.?" dataDxfId="5">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r376db28f5b7c43279bb964be0e2eb715"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="127" xr3:uid="{00000000-0010-0000-0000-00007F000000}" name="List all Contract Agreement Exhibit / Appendix (Letter / Number /Name)" dataDxfId="4">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r397e92fd4068432a9d1dc76da74eadb4"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="128" xr3:uid="{00000000-0010-0000-0000-000080000000}" name="Are there any Contract Agreement / Specifications Containing BIM Requirements?" dataDxfId="3">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r55c798a5e6114b1999261746814bb5cc"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="123" xr3:uid="{00000000-0010-0000-0000-00007B000000}" name="Hazardous Materials - IMC is Only Responsible Content Created by Us or our Subcontractors" dataDxfId="8"/>
+    <tableColumn id="124" xr3:uid="{00000000-0010-0000-0000-00007C000000}" name="Hazardous Materials - IMC is Entitled to Stop Work, and Recover Cost for Delay for_x000a_  Encountered Hazardous Material" dataDxfId="7"/>
+    <tableColumn id="125" xr3:uid="{00000000-0010-0000-0000-00007D000000}" name="What is the Labor?" dataDxfId="6"/>
+    <tableColumn id="126" xr3:uid="{00000000-0010-0000-0000-00007E000000}" name="Is IMC Responsible to Recover Delay (Cost &amp; Schedule) for labor related work stoppage;_x000a_  strike etc.?" dataDxfId="5"/>
+    <tableColumn id="127" xr3:uid="{00000000-0010-0000-0000-00007F000000}" name="List all Contract Agreement Exhibit / Appendix (Letter / Number /Name)" dataDxfId="4"/>
+    <tableColumn id="128" xr3:uid="{00000000-0010-0000-0000-000080000000}" name="Are there any Contract Agreement / Specifications Containing BIM Requirements?" dataDxfId="3"/>
     <tableColumn id="129" xr3:uid="{00000000-0010-0000-0000-000081000000}" name="What is the Cyber Indemnification / Hacking Article #?" dataDxfId="2"/>
-    <tableColumn id="130" xr3:uid="{00000000-0010-0000-0000-000082000000}" name="What are the Cyber Indemnification / Hacking Article Terms &amp; Conditions?" dataDxfId="1">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="r1c80022f839648268632e2286e41c2d8"/>
-        </ext>
-      </extLst>
-    </tableColumn>
-    <tableColumn id="131" xr3:uid="{2AAF5914-0F8A-4F29-AAE6-511C69C3C364}" name="Who is Responsible to pay the Builders Risk Deductible? (May Vary Depending on Amount)" dataDxfId="0">
-      <extLst>
-        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
-          <xlmsforms:question id="rd5a286cdaf3946cb873be3873bc184b7"/>
-        </ext>
-      </extLst>
-    </tableColumn>
+    <tableColumn id="130" xr3:uid="{00000000-0010-0000-0000-000082000000}" name="What are the Cyber Indemnification / Hacking Article Terms &amp; Conditions?" dataDxfId="1"/>
+    <tableColumn id="131" xr3:uid="{2AAF5914-0F8A-4F29-AAE6-511C69C3C364}" name="Who is Responsible to pay the Builders Risk Deductible? (May Vary Depending on Amount)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-  <extLst>
-    <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="P0YbIax95UuNtfh0kfaJ6QenDOCl-mFJov_kZV9wTP1UMVBETVBIQjNOUjlFVEUxQjE4MFVUSzBFSCQlQCN0PWcu" isFormConnected="1" maxResponseId="27" latestEventMarker="9">
-        <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rc2901229e6604efb8202cde185cec144</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r216255fe8cbc4d08ab0109f4de1d61b7</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r603600d87fc5401c8e50b4b82ee0e1b4</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r50d5dcc2b0b8467cbfa057ae78eb727b</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r71eec1ad3095454489076c8df8dd6f2d</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r98a6045c74294501a236c2d58930a2d1</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r5d645ce804e343f289e48c56f820ade9</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r2762b1bd4a7e46ee8aea16ea651f08cb</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r31f357e6c7814e978a1190d0dea30125</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r7befd93a2b044ddcb732af34021a7d68</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r511f20b7ad754365b8911145766f7d2c</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r04c110c6f3904c37894eec3af1b6f577</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r9649ee9242b2466f860eab1f1ab1ec69</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r88d51b5c8aad479d846e9270635a68dd</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r7506d7a2568f4cbc801da6dfd331073b</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>red658e215a034f4a9b4e4d0669b99d64</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r55ecd76cb2f8456c86d9f98841c17b1f</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r3aefc1d090a74439b684bb4b245b2177</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r0dd5ea5075534da8adc5163fc641e754</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rb9f3e9f03f824bac8b97ad79309b8b80</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r61e13bffea00487a89561a5286eddd70</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>ra0b8f43bd5a0458397bca3de86c47df1</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r4bbab4541b2847df9ac326d5844756d5</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r5a009cdb311b4b30bc983bcd6a2c5063</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r376db28f5b7c43279bb964be0e2eb715</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r20892b4c7cd44a4ab993418747b11a00</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>re35f6e8c39504df5a53ab299d2c75388</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>raa0a22f6e8c843569c9f103702978d9c</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r123dd14384f449e0ae91d811f71dad3e</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r94b71574e77144a9944acab61e704546</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r86c1b7203b3443f3be9c09a62ec8a2dd</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r71be6f0b174849f0b3c027cae6320fed</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rbd05295cc26a4fdd89fed946070ef8fc</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r219eb35008dd426db1f843a8ca13cd40</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r3e1f9ae94afa448a9418b710cb752f34</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r13b23d7a98b24697833e7b4706ee64df</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rc8a478ec1f45406a9068cf17f0e292d9</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>ref2cc6ee8621439892c97520c392e379</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r79ec9c8349034fa19d9d4e7174300ef8</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r6096f99c96944892a8742a600d7a25c9</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r16fbd2d0ede144398dc1d38017db246f</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rb29a12d680724ea7a57805d41ba7a872</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rf87b2a6e53a644849cfb2d142aa857d2</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>responderName</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rcf60812b97f642489be7187347eecf59</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r234a80e39db04a179f4e69d1f7f8305a</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>re5de246da8c448649597351cc4ac3e63</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r0e8520abe8c34ec0b67941171a4f7ad3</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r62018dadbca944eb8e13d572a5e25a92</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r91aa4272d0e8428ab83090d2151968e1</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r90bbdc8c6ce248a8aef415ae2a0a0bc6</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rf51502d08e1f4893832e976c8314d940</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r88c463a257ca4ac591b3b83ba8b5e495</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r397e92fd4068432a9d1dc76da74eadb4</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rcb39888485954b849ec25be717540429</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r2c27a4dfe6254b67a6a612103e619369</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r1ba7d730cb1d45cfb45f41fdd8d3f726</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r79d8d8378ee14f61a0aca947618aa45e</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r765d687918fb4bd388cd9593d18256bf</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rd5a286cdaf3946cb873be3873bc184b7</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rfbb7e9f167b94f2092dc0076844d8ba5</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r64b0f1d30e4043d1b039a10f86a00c06</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rddb08ff6ba1a4f22801cbd84cd68b9ff</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>re8020cd41e464042bec4618f513425f6</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r8f48763501c141cabcba9ccb9f7387b8</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rc8125195f5784cd0bcbe5834f31ba726</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r6b642609bbd2483496535f5ea4426402</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r7d90da3b6d0d4d5ab58194bafa660753</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r61312d8a3bf241b595a8a7cea92d7d7c</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r4ee458eeafc24c60981e7abfa3f60afc</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rbc70f0e67c2546ce991f8ceda7d12e27</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r1aef87de3aaa46b292efd902412fb1db</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rccc43ba04ce8481d82e5bbfa65d5efc8</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r69ddd5267a474d7fbf1ef4a31f0b343a</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r2b239e19bc72478f9703cfb6ea697743</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r1150fbd8e5ce40bd9ae6b4d3aca9c087</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r9222b568c0764e8b9f86561d7612dc80</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r75c08cbdffb9486eba28ecf67b79f977</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>responder</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r6a2252e44d17494baf7280077a8d7048</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r1e4222322f8a4b3290b5994aa0c4d432</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r91aacfed7c034922963019a3a708273e</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r333878a557e64604a2416d5356acb191</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r651c21d8cd044857bc5d4c2e6f1f15f7</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r53ef0168697245aea3523acf623b5b6e</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r36e4d147820949b0a778dc56a7b1b9d6</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r7c3dc7565df04de5a818045f10cebda4</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r665a7ea397a34d568aac3d8e8420000f</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rf250282fa9f047f292532a1f38dd6422</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r3f1689564d114dc1a62c0287b4a19e3f</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r421f93c42ecd4034968430d5904a832d</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r68c6e076211347e6b7373b3eabe809fa</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rb99c4ad090964c53a9848257e1b6ec86</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r8cd57f4b8b7c4f3e9383f6cc22643e5f</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rb7970e13cb2c4da085a4bde4a67b4cf5</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r1c80022f839648268632e2286e41c2d8</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r29fa239322c4423eaf7df132373c4df6</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>ra94986dd41e9411786bd6a9547d5dce9</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r55c798a5e6114b1999261746814bb5cc</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>r99a0cc669ecc4fdfba741c1754b46757</xlmsforms:syncedQuestionId>
-        <xlmsforms:syncedQuestionId>rbbec339b56db4500836dd7699a6a717e</xlmsforms:syncedQuestionId>
-      </xlmsforms:msForm>
-    </ext>
-  </extLst>
 </table>
 </file>
 
@@ -6979,17 +6364,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:DU28"/>
-  <sheetFormatPr defaultRowHeight="100.05" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="99.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="2" max="21" width="20" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="44.44140625" customWidth="1"/>
+    <col min="22" max="22" width="44.42578125" customWidth="1"/>
     <col min="23" max="124" width="20" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="28.5546875" customWidth="1"/>
+    <col min="125" max="125" width="28.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -7364,9 +6750,9 @@
         <v>130</v>
       </c>
     </row>
-    <row r="2" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
+    <row r="2" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1315</v>
       </c>
       <c r="B2">
         <v>8</v>
@@ -7668,9 +7054,9 @@
         <v>816</v>
       </c>
     </row>
-    <row r="3" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
+    <row r="3" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1317</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -8027,9 +7413,9 @@
       <c r="DT3" s="3"/>
       <c r="DU3" s="3"/>
     </row>
-    <row r="4" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
+    <row r="4" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1318</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -8399,9 +7785,9 @@
       </c>
       <c r="DU4" s="3"/>
     </row>
-    <row r="5" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
+    <row r="5" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1319</v>
       </c>
       <c r="B5">
         <v>23</v>
@@ -8696,9 +8082,9 @@
         <v>384</v>
       </c>
     </row>
-    <row r="6" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
+    <row r="6" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>1320</v>
       </c>
       <c r="B6">
         <v>11</v>
@@ -8997,9 +8383,9 @@
         <v>384</v>
       </c>
     </row>
-    <row r="7" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
+    <row r="7" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>1321</v>
       </c>
       <c r="B7">
         <v>15</v>
@@ -9301,9 +8687,9 @@
         <v>508</v>
       </c>
     </row>
-    <row r="8" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>7</v>
+    <row r="8" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>1322</v>
       </c>
       <c r="B8">
         <v>9</v>
@@ -9607,9 +8993,9 @@
         <v>763</v>
       </c>
     </row>
-    <row r="9" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>8</v>
+    <row r="9" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>1323</v>
       </c>
       <c r="B9">
         <v>5</v>
@@ -9979,9 +9365,9 @@
       </c>
       <c r="DU9" s="3"/>
     </row>
-    <row r="10" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>17</v>
+    <row r="10" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>1324</v>
       </c>
       <c r="B10">
         <v>4</v>
@@ -10319,9 +9705,9 @@
       </c>
       <c r="DU10" s="3"/>
     </row>
-    <row r="11" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>18</v>
+    <row r="11" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>1325</v>
       </c>
       <c r="B11">
         <v>19</v>
@@ -10623,9 +10009,9 @@
         <v>344</v>
       </c>
     </row>
-    <row r="12" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>9</v>
+    <row r="12" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1326</v>
       </c>
       <c r="B12">
         <v>7</v>
@@ -10929,9 +10315,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="13" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>10</v>
+    <row r="13" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>1327</v>
       </c>
       <c r="B13">
         <v>14</v>
@@ -11235,9 +10621,9 @@
         <v>570</v>
       </c>
     </row>
-    <row r="14" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>11</v>
+    <row r="14" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>1328</v>
       </c>
       <c r="B14">
         <v>24</v>
@@ -11520,9 +10906,9 @@
       <c r="DT14" s="3"/>
       <c r="DU14" s="3"/>
     </row>
-    <row r="15" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>19</v>
+    <row r="15" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>1329</v>
       </c>
       <c r="B15">
         <v>13</v>
@@ -11822,9 +11208,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>20</v>
+    <row r="16" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>1330</v>
       </c>
       <c r="B16">
         <v>10</v>
@@ -12128,9 +11514,9 @@
         <v>575</v>
       </c>
     </row>
-    <row r="17" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>21</v>
+    <row r="17" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>1331</v>
       </c>
       <c r="B17">
         <v>16</v>
@@ -12434,9 +11820,9 @@
         <v>442</v>
       </c>
     </row>
-    <row r="18" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>12</v>
+    <row r="18" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1332</v>
       </c>
       <c r="B18">
         <v>12</v>
@@ -12738,9 +12124,9 @@
         <v>619</v>
       </c>
     </row>
-    <row r="19" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>22</v>
+    <row r="19" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>1333</v>
       </c>
       <c r="B19">
         <v>17</v>
@@ -13044,9 +12430,9 @@
         <v>436</v>
       </c>
     </row>
-    <row r="20" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>13</v>
+    <row r="20" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>1334</v>
       </c>
       <c r="B20">
         <v>18</v>
@@ -13350,9 +12736,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="21" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>14</v>
+    <row r="21" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>1335</v>
       </c>
       <c r="B21">
         <v>21</v>
@@ -13644,9 +13030,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="22" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>23</v>
+    <row r="22" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1336</v>
       </c>
       <c r="B22">
         <v>26</v>
@@ -13948,9 +13334,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="23" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>22</v>
+    <row r="23" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>1333</v>
       </c>
       <c r="B23">
         <v>22</v>
@@ -14254,9 +13640,9 @@
         <v>181</v>
       </c>
     </row>
-    <row r="24" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>24</v>
+    <row r="24" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>1337</v>
       </c>
       <c r="B24">
         <v>20</v>
@@ -14530,9 +13916,9 @@
         <v>289</v>
       </c>
     </row>
-    <row r="25" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>16</v>
+    <row r="25" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>1338</v>
       </c>
       <c r="B25">
         <v>25</v>
@@ -14836,9 +14222,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="26" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>25</v>
+    <row r="26" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>1339</v>
       </c>
       <c r="B26">
         <v>27</v>
@@ -15140,7 +14526,7 @@
         <v>1311</v>
       </c>
     </row>
-    <row r="27" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27">
         <v>1</v>
       </c>
@@ -15439,7 +14825,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="28" spans="1:125" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:125" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28">
         <v>2</v>
       </c>
@@ -15471,9 +14857,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E4E13AB-34AB-4626-A0E7-12F0F3215D86}">
   <dimension ref="A1:EA1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:131" ht="244.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:131" ht="255" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -15876,13 +15262,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD8B569-1632-4BF1-AFBD-24E1F24E3B55}">
   <dimension ref="A1:B131"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="99.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.109375" customWidth="1"/>
+    <col min="1" max="1" width="99.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -15890,7 +15276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -15898,7 +15284,7 @@
         <v>45041.634212962999</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -15906,7 +15292,7 @@
         <v>45041.636909722198</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -15914,7 +15300,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -15922,7 +15308,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -15930,7 +15316,7 @@
         <v>45041</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -15938,7 +15324,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -15946,12 +15332,12 @@
         <v>1101</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -15959,127 +15345,127 @@
         <v>1102</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -16087,7 +15473,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -16095,7 +15481,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -16103,7 +15489,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -16111,7 +15497,7 @@
         <v>1104</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -16119,7 +15505,7 @@
         <v>1105</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -16127,7 +15513,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -16135,7 +15521,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -16143,7 +15529,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -16151,7 +15537,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -16159,7 +15545,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -16167,7 +15553,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -16175,7 +15561,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>46</v>
       </c>
@@ -16183,7 +15569,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -16191,7 +15577,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -16199,7 +15585,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>49</v>
       </c>
@@ -16207,7 +15593,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>50</v>
       </c>
@@ -16215,7 +15601,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>51</v>
       </c>
@@ -16223,7 +15609,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>52</v>
       </c>
@@ -16231,7 +15617,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>53</v>
       </c>
@@ -16239,7 +15625,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>54</v>
       </c>
@@ -16247,7 +15633,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>55</v>
       </c>
@@ -16255,7 +15641,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>56</v>
       </c>
@@ -16263,7 +15649,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>57</v>
       </c>
@@ -16271,7 +15657,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>58</v>
       </c>
@@ -16279,7 +15665,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -16287,7 +15673,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>60</v>
       </c>
@@ -16295,7 +15681,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>61</v>
       </c>
@@ -16303,7 +15689,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>62</v>
       </c>
@@ -16311,7 +15697,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>63</v>
       </c>
@@ -16319,7 +15705,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>64</v>
       </c>
@@ -16327,7 +15713,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>65</v>
       </c>
@@ -16335,7 +15721,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>66</v>
       </c>
@@ -16343,7 +15729,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>67</v>
       </c>
@@ -16351,7 +15737,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>68</v>
       </c>
@@ -16359,7 +15745,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>69</v>
       </c>
@@ -16367,7 +15753,7 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -16375,7 +15761,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -16383,7 +15769,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>72</v>
       </c>
@@ -16391,7 +15777,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -16399,7 +15785,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>74</v>
       </c>
@@ -16407,7 +15793,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>75</v>
       </c>
@@ -16415,7 +15801,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>76</v>
       </c>
@@ -16423,7 +15809,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>77</v>
       </c>
@@ -16431,7 +15817,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>78</v>
       </c>
@@ -16439,7 +15825,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>79</v>
       </c>
@@ -16447,7 +15833,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>80</v>
       </c>
@@ -16455,7 +15841,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>81</v>
       </c>
@@ -16463,7 +15849,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>82</v>
       </c>
@@ -16471,7 +15857,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -16479,7 +15865,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>84</v>
       </c>
@@ -16487,7 +15873,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>85</v>
       </c>
@@ -16495,7 +15881,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>86</v>
       </c>
@@ -16503,7 +15889,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>87</v>
       </c>
@@ -16511,7 +15897,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>88</v>
       </c>
@@ -16519,7 +15905,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>89</v>
       </c>
@@ -16527,7 +15913,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>90</v>
       </c>
@@ -16535,7 +15921,7 @@
         <v>1114</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>91</v>
       </c>
@@ -16543,7 +15929,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>92</v>
       </c>
@@ -16551,7 +15937,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>93</v>
       </c>
@@ -16559,7 +15945,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>94</v>
       </c>
@@ -16567,7 +15953,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>95</v>
       </c>
@@ -16575,7 +15961,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>96</v>
       </c>
@@ -16583,7 +15969,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>97</v>
       </c>
@@ -16591,7 +15977,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>98</v>
       </c>
@@ -16599,7 +15985,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>99</v>
       </c>
@@ -16607,7 +15993,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>100</v>
       </c>
@@ -16615,7 +16001,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>101</v>
       </c>
@@ -16623,7 +16009,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>102</v>
       </c>
@@ -16631,7 +16017,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>103</v>
       </c>
@@ -16639,7 +16025,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>104</v>
       </c>
@@ -16647,7 +16033,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>105</v>
       </c>
@@ -16655,7 +16041,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>106</v>
       </c>
@@ -16663,7 +16049,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>107</v>
       </c>
@@ -16671,7 +16057,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>108</v>
       </c>
@@ -16679,7 +16065,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>109</v>
       </c>
@@ -16687,7 +16073,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>110</v>
       </c>
@@ -16695,7 +16081,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>111</v>
       </c>
@@ -16703,7 +16089,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>112</v>
       </c>
@@ -16711,7 +16097,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>113</v>
       </c>
@@ -16719,7 +16105,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>114</v>
       </c>
@@ -16727,7 +16113,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>115</v>
       </c>
@@ -16735,7 +16121,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>116</v>
       </c>
@@ -16743,7 +16129,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>117</v>
       </c>
@@ -16751,7 +16137,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>118</v>
       </c>
@@ -16759,7 +16145,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>119</v>
       </c>
@@ -16767,7 +16153,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>120</v>
       </c>
@@ -16775,7 +16161,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>121</v>
       </c>
@@ -16783,7 +16169,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>122</v>
       </c>
@@ -16791,7 +16177,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="124" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
         <v>123</v>
       </c>
@@ -16799,7 +16185,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>124</v>
       </c>
@@ -16807,7 +16193,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="126" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
         <v>125</v>
       </c>
@@ -16815,7 +16201,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>126</v>
       </c>
@@ -16823,7 +16209,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>127</v>
       </c>
@@ -16831,7 +16217,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>128</v>
       </c>
@@ -16839,7 +16225,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>129</v>
       </c>
@@ -16847,7 +16233,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>130</v>
       </c>
@@ -16860,24 +16246,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1313</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>17</v>
       </c>
@@ -16889,15 +16275,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003DB2C4F0D349EA4DA416001B9762A470" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="68a410158b457edd41b7d9bac17783a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d5146b02-3afe-4095-87ab-12a3f19b7856" xmlns:ns3="91ed1f9b-b396-41d7-b6e3-0a27034e321f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cc0b54de1222dd8245870c18ba2bd9f2" ns2:_="" ns3:_="">
     <xsd:import namespace="d5146b02-3afe-4095-87ab-12a3f19b7856"/>
@@ -17158,6 +16535,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -17170,14 +16556,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0EAC4F8-29CD-4182-9B14-26BE12CBEAFD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7C1E539-B583-4017-9791-776218F7EE03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17196,13 +16574,27 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0EAC4F8-29CD-4182-9B14-26BE12CBEAFD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{184CF6A5-DA6E-4508-84ED-4C1A57F2C98D}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="91ed1f9b-b396-41d7-b6e3-0a27034e321f"/>
     <ds:schemaRef ds:uri="d5146b02-3afe-4095-87ab-12a3f19b7856"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>